<commit_message>
update next cosmetic and next cosmetic artist
</commit_message>
<xml_diff>
--- a/public/sheets/dunkbin_next_cosmetic_info.xlsx
+++ b/public/sheets/dunkbin_next_cosmetic_info.xlsx
@@ -412,13 +412,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Fly Agaric Hat + Minecraft soil</v>
+        <v>Hachiware</v>
       </c>
       <c r="B2">
-        <v>1679</v>
+        <v>1672</v>
       </c>
       <c r="C2" t="str">
-        <v>miczupl</v>
+        <v>superpapipig</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
2026-10-14 update next cosmetic info
</commit_message>
<xml_diff>
--- a/public/sheets/dunkbin_next_cosmetic_info.xlsx
+++ b/public/sheets/dunkbin_next_cosmetic_info.xlsx
@@ -412,13 +412,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Chit</v>
+        <v>Hat hat</v>
       </c>
       <c r="B2">
-        <v>1718</v>
+        <v>1428</v>
       </c>
       <c r="C2" t="str">
-        <v>maito1794</v>
+        <v>snekiecr8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
2026-10-15 update next cosmetic info
</commit_message>
<xml_diff>
--- a/public/sheets/dunkbin_next_cosmetic_info.xlsx
+++ b/public/sheets/dunkbin_next_cosmetic_info.xlsx
@@ -412,13 +412,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Hat hat</v>
+        <v>Perry the Platypus Hat</v>
       </c>
       <c r="B2">
-        <v>1428</v>
+        <v>951</v>
       </c>
       <c r="C2" t="str">
-        <v>snekiecr8</v>
+        <v>any_one_plz</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
2026-10-17 update next cosmetic info
</commit_message>
<xml_diff>
--- a/public/sheets/dunkbin_next_cosmetic_info.xlsx
+++ b/public/sheets/dunkbin_next_cosmetic_info.xlsx
@@ -412,13 +412,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Perry the Platypus Hat</v>
+        <v>Ooze Head</v>
       </c>
       <c r="B2">
-        <v>951</v>
+        <v>1151</v>
       </c>
       <c r="C2" t="str">
-        <v>any_one_plz</v>
+        <v>clown_noes666</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
2026-10-18 update next cosmetic info
</commit_message>
<xml_diff>
--- a/public/sheets/dunkbin_next_cosmetic_info.xlsx
+++ b/public/sheets/dunkbin_next_cosmetic_info.xlsx
@@ -412,13 +412,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Ooze Head</v>
+        <v>Bora Headpiece</v>
       </c>
       <c r="B2">
-        <v>1151</v>
+        <v>1399</v>
       </c>
       <c r="C2" t="str">
-        <v>clown_noes666</v>
+        <v>flippy826</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
2026-10-21 update next cosmetic info
</commit_message>
<xml_diff>
--- a/public/sheets/dunkbin_next_cosmetic_info.xlsx
+++ b/public/sheets/dunkbin_next_cosmetic_info.xlsx
@@ -412,13 +412,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Bora Headpiece</v>
+        <v>Dr. Beanies</v>
       </c>
       <c r="B2">
-        <v>1399</v>
+        <v>1697</v>
       </c>
       <c r="C2" t="str">
-        <v>flippy826</v>
+        <v>uplift3ntree</v>
       </c>
     </row>
   </sheetData>

</xml_diff>